<commit_message>
test(hw03): execute GUI checklist and report defects
</commit_message>
<xml_diff>
--- a/hw/hw3/23127334_HW03_AI_GUIUsability_TBD/task-1-gui-checklist/gui-checklist-v1-reviewed.xlsx
+++ b/hw/hw3/23127334_HW03_AI_GUIUsability_TBD/task-1-gui-checklist/gui-checklist-v1-reviewed.xlsx
@@ -580,11 +580,31 @@
           <t>PASS if exactly one h1 identifies the page as Đăng nhập; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Found 0 h1 elements; visible h2 text is "Đăng Ký".</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-001.png</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -632,11 +652,31 @@
           <t>PASS if uI is consistently Vietnamese except accepted technical terms; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-language labels are visible: "Username" and "Sign In".</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-002.png</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-001</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -684,9 +724,21 @@
           <t>PASS if all elements align with adequate spacing and no overlap; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>No overlap detected in the desktop Login card.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr"/>
     </row>
@@ -736,9 +788,21 @@
           <t>PASS if no clipping or horizontal page scroll; targets remain usable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>No horizontal overflow at 320 px (320/320).</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr"/>
     </row>
@@ -788,11 +852,31 @@
           <t>PASS if normal text ≥4.5:1 and meaningful UI components ≥3:1; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>The light-blue “Quên mật khẩu?” link (#3B82F6 on white) is approximately 3.68:1, below WCAG AA 4.5:1 for normal text.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Computed-color contrast measurement in Chromium.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-005.png</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-002</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -840,11 +924,31 @@
           <t>PASS if primary controls are at least 44×44 CSS px or equivalently usable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Targets below 44×44: EShop 70×32; Giỏ hàng 64×24; Đăng nhập 78×24; Đăng ký 58×24; INPUT 382×42; INPUT 382×42; Quên mật khẩu? 102×19; Sign In 382×40; Đăng ký ngay 85×19.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-006.png</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-002</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -892,11 +996,31 @@
           <t>PASS if input type is email and native validation rejects malformed format; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Email/Username control uses type="text".</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-007.png</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-003</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -944,11 +1068,31 @@
           <t>PASS if control uses password type and characters are masked; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Password control uses type="text" and exposes the entered value.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-008.png</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-003</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -996,11 +1140,31 @@
           <t>PASS if both mandatory labels include a visible required marker; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Required markers are absent from labels: Username | Mật khẩu.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-009.png</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-004</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1048,11 +1212,31 @@
           <t>PASS if each label focuses its input and supplies the accessible name; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Login labels have no for/id association and do not wrap their inputs.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-010.png</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-004</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1100,11 +1284,31 @@
           <t>PASS if visible validation identifies both required fields near their controls; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>No two-field visible validation summary/inline messages; detected 0 explicit error elements.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-011A.png</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-004</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1152,11 +1356,31 @@
           <t>PASS if focus order is Email, Password, Forgot password, Submit, Register; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Observed focus order: EShopGiỏ hàngĐăng nhậpĐăng kýĐăng KýUsernameMật khẩuQuên mật khẩu?Sign InChưa có tài khoản? Đăng ký ngay© 2026 EShop SUT. Dành cho mục đích kiểm thử. → Sign In → EShop → Giỏ hàng → Đăng nhập.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-013.png</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-005</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1204,9 +1428,21 @@
           <t>PASS if a persistent, high-contrast focus indicator is visible; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Every tested interactive element exposes a focus indicator.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr"/>
     </row>
@@ -1256,11 +1492,31 @@
           <t>PASS if email and current password can be filled into the correct fields; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Autocomplete tokens are [null,null] instead of email/current-password.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-020.png</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-003</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1308,9 +1564,21 @@
           <t>PASS if no content or focus indicator is clipped; reflow remains usable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No horizontal clipping detected at 200% page scale.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
     </row>
@@ -1360,9 +1628,21 @@
           <t>PASS if no text, control, or focus indicator overlaps or becomes unreachable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Exploratory RTL run produced no overlap or unreachable controls.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr"/>
     </row>
@@ -1412,11 +1692,31 @@
           <t>PASS if the submit control visibly indicates a pending state and prevents repeated activation; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr"/>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Submit remains enabled and shows no pending indicator during repeated activation.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-024A.png</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-006</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1464,9 +1764,21 @@
           <t>PASS if every row visibly contains all four FR-11 fields; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>5 rows each display ID, date, total, and status.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
     </row>
@@ -1516,9 +1828,21 @@
           <t>PASS if orders are sorted newest first or sorting is clearly provided; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Order IDs displayed newest first: 5, 4, 3, 2, 1.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
     </row>
@@ -1568,11 +1892,31 @@
           <t>PASS if values use Vietnamese thousands separators and ₫ consistently; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Non-Vietnamese/ambiguous currency format: 550,000 ₫, 450,000 ₫, 350,000 ₫, 250,000 ₫, 150,000 ₫.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-005.png</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-007</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1620,11 +1964,31 @@
           <t>PASS if day, month, and year are unambiguous and consistent; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Dates render with browser-default US ordering such as 7/26/2026 instead of deterministic Vietnamese day/month/year formatting.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Observed across all five seeded order rows in Chromium.</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-006.png</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-007</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1672,9 +2036,21 @@
           <t>PASS if every backend state maps to the specified Vietnamese meaning; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>All five Vietnamese statuses displayed.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr"/>
     </row>
@@ -1724,9 +2100,21 @@
           <t>PASS if states are consistently distinguishable and remain readable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Each visible status has readable text and a distinct badge color.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr"/>
     </row>
@@ -1776,11 +2164,31 @@
           <t>PASS if a confirmation dialog names the consequence before mutation; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>No confirmation dialog; cancel request executes immediately and only a result alert appears.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-010.png</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-008</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1828,11 +2236,31 @@
           <t>PASS if action and dialog work without pointer and focus returns logically; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard activates cancel but no confirmation dialog exists.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-011.png</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-008</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1880,11 +2308,31 @@
           <t>PASS if profile/order history entry is clearly discoverable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Only profile greeting "Chào, Test User" leads to history; Order History is not named in navigation.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-012.png</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-009</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1932,11 +2380,31 @@
           <t>PASS if current destination is visually and programmatically indicated; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Current Profile/History navigation has no aria-current or active-state marker.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-013.png</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-009</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1984,11 +2452,31 @@
           <t>PASS if a non-blocking loading indicator appears until data resolves; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>No loading indicator during a 1.2-second delayed order request.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-016.png</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-010</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2036,9 +2524,21 @@
           <t>PASS if readable text communicates every state independently of color; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Every status badge includes a Vietnamese text label independent of color.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr"/>
     </row>
@@ -2088,11 +2588,31 @@
           <t>PASS if table has caption/context, column headers, and correct associations; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Table has 5 column headers but 0 caption elements.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-019.png</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-011</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2140,11 +2660,31 @@
           <t>PASS if table reflows or provides controlled scroll without page-wide clipping; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Order table causes page-wide horizontal clipping at 320 px.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-020.png</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-012</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2192,11 +2732,31 @@
           <t>PASS if labels, totals, status, and actions remain visible and usable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Order History clips horizontally at 200% scale.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-021.png</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-012</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2244,11 +2804,31 @@
           <t>PASS if clear error and recovery action appear; empty-state message is not shown; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>API failure is shown as "Lịch sử đơn hàng" with no retry action.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-022.png</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-010</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2296,9 +2876,21 @@
           <t>PASS if visible feedback clearly communicates success or failure without ambiguity; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Visible result alert: "Hủy đơn thành công!".</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr"/>
     </row>
@@ -2348,11 +2940,31 @@
           <t>PASS if each error is visible, names the affected field, and is programmatically associated with that field; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>No explicit inline error, error summary, aria-invalid, or aria-describedby association is rendered for either required field.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>DOM and accessibility-attribute inspection after empty submission.</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-025.png</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-004</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2400,11 +3012,31 @@
           <t>PASS if the complete error is announced and focus remains at a logical control; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>The dynamically inserted credential error has no role=alert, aria-live, or equivalent live-region semantics.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>DOM inspection after failed credential submission.</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-L-026.png</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-004</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2452,9 +3084,21 @@
           <t>PASS if every focused control and its focus indicator remain at least partially visible; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>All focused Login controls remain inside the viewport at desktop/mobile sizes.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
     </row>
@@ -2504,9 +3148,21 @@
           <t>PASS if no label, link, input value, error, or button text is clipped or overlaps; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>No horizontal overflow with WCAG text-spacing overrides.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr"/>
     </row>
@@ -2556,9 +3212,21 @@
           <t>PASS if the same controls and content remain available and usable in both orientations; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>All Login controls remained available in portrait 390×844 and landscape 844×390.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
     </row>
@@ -2608,9 +3276,21 @@
           <t>PASS if all text, controls, focus indicators, and errors remain visible and distinguishable; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Exploratory dark preference run retained visible Login content and controls.</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr"/>
     </row>
@@ -2660,11 +3340,31 @@
           <t>PASS if the table exposes a concise accessible caption identifying it as order history; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>The Order History table has no caption and exposes no dedicated accessible table name.</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>DOM/table semantic inspection.</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-025.png</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-011</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2712,9 +3412,21 @@
           <t>PASS if each row is announced in the visible column order without detached or repeated values; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr"/>
-      <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Requires a real screen-reader reading-order check at desktop and mobile widths.</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Requires manual assistive-technology or OS-level execution.</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
     </row>
@@ -2764,11 +3476,31 @@
           <t>PASS if focus enters the dialog, cycles within it, and returns to the invoking control after close; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
-      <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>No cancel confirmation dialog exists, so dialog focus containment/return cannot be satisfied.</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-027.png</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-008</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2816,11 +3548,31 @@
           <t>PASS if any required horizontal scrolling is confined to the table region and surrounding page content reflows; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr"/>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
-      <c r="M45" s="2" t="inlineStr"/>
-      <c r="N45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Wide table has no localized horizontal-scroll container.</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Observed during automated Playwright execution; see linked failure screenshot.</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>failed-screenshots/GUI-O-028.png</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>BUG-GUI-012</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2868,9 +3620,21 @@
           <t>PASS if the updated state or confirmation is announced without requiring focus movement; otherwise FAIL</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Requires a real screen-reader status-message announcement check.</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Requires manual assistive-technology or OS-level execution.</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
test(hw3): update Task 1 bug report and GitHub issue links
</commit_message>
<xml_diff>
--- a/hw/hw3/23127334_HW03_AI_GUIUsability_TBD/task-1-gui-checklist/gui-checklist-v1-reviewed.xlsx
+++ b/hw/hw3/23127334_HW03_AI_GUIUsability_TBD/task-1-gui-checklist/gui-checklist-v1-reviewed.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-001</t>
+          <t>BUG-GUI-001 — https://github.com/ThanhDang-Vn/software-testing/issues/18</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-001</t>
+          <t>BUG-GUI-001 — https://github.com/ThanhDang-Vn/software-testing/issues/18</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-002</t>
+          <t>BUG-GUI-002 — https://github.com/ThanhDang-Vn/software-testing/issues/19</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-002</t>
+          <t>BUG-GUI-002 — https://github.com/ThanhDang-Vn/software-testing/issues/19</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-003</t>
+          <t>BUG-GUI-003 — https://github.com/ThanhDang-Vn/software-testing/issues/20</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-003</t>
+          <t>BUG-GUI-003 — https://github.com/ThanhDang-Vn/software-testing/issues/20</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-004</t>
+          <t>BUG-GUI-004 — https://github.com/ThanhDang-Vn/software-testing/issues/21</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-004</t>
+          <t>BUG-GUI-004 — https://github.com/ThanhDang-Vn/software-testing/issues/21</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-004</t>
+          <t>BUG-GUI-004 — https://github.com/ThanhDang-Vn/software-testing/issues/21</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-005</t>
+          <t>BUG-GUI-005 — https://github.com/ThanhDang-Vn/software-testing/issues/22</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-003</t>
+          <t>BUG-GUI-003 — https://github.com/ThanhDang-Vn/software-testing/issues/20</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-006</t>
+          <t>BUG-GUI-006 — https://github.com/ThanhDang-Vn/software-testing/issues/23</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-007</t>
+          <t>BUG-GUI-007 — https://github.com/ThanhDang-Vn/software-testing/issues/24</t>
         </is>
       </c>
     </row>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-007</t>
+          <t>BUG-GUI-007 — https://github.com/ThanhDang-Vn/software-testing/issues/24</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-008</t>
+          <t>BUG-GUI-008 — https://github.com/ThanhDang-Vn/software-testing/issues/25</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-008</t>
+          <t>BUG-GUI-008 — https://github.com/ThanhDang-Vn/software-testing/issues/25</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-009</t>
+          <t>BUG-GUI-009 — https://github.com/ThanhDang-Vn/software-testing/issues/26</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-009</t>
+          <t>BUG-GUI-009 — https://github.com/ThanhDang-Vn/software-testing/issues/26</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-010</t>
+          <t>BUG-GUI-010 — https://github.com/ThanhDang-Vn/software-testing/issues/27</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-011</t>
+          <t>BUG-GUI-011 — https://github.com/ThanhDang-Vn/software-testing/issues/28</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-012</t>
+          <t>BUG-GUI-012 — https://github.com/ThanhDang-Vn/software-testing/issues/29</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2754,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-012</t>
+          <t>BUG-GUI-012 — https://github.com/ThanhDang-Vn/software-testing/issues/29</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-010</t>
+          <t>BUG-GUI-010 — https://github.com/ThanhDang-Vn/software-testing/issues/27</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-004</t>
+          <t>BUG-GUI-004 — https://github.com/ThanhDang-Vn/software-testing/issues/21</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-004</t>
+          <t>BUG-GUI-004 — https://github.com/ThanhDang-Vn/software-testing/issues/21</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-011</t>
+          <t>BUG-GUI-011 — https://github.com/ThanhDang-Vn/software-testing/issues/28</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-008</t>
+          <t>BUG-GUI-008 — https://github.com/ThanhDang-Vn/software-testing/issues/25</t>
         </is>
       </c>
     </row>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>BUG-GUI-012</t>
+          <t>BUG-GUI-012 — https://github.com/ThanhDang-Vn/software-testing/issues/29</t>
         </is>
       </c>
     </row>

</xml_diff>